<commit_message>
[EC 09/09] Mestra mantida como v4.3.4 por decisao do LEO; v4.3.5 removida
O LEO reafirmou a preferencia por manter o nome v4_3_4 depois de o custo ter
sido apresentado. Feito: o conteudo de hoje sobrescreve a v4_3_4 e a v4_3_5 sai
do repositorio. Referencias canonicas do CLAUDE.md voltam para v4.3.4.

O arquivo tambem ganhou o numero do pedido na linha da devolucao.

O changelog abre com o aviso de que v4.3.4 designa dois conteudos e traz o
comando git show para recuperar o de 08/09, que segue preservado no historico.
Registra tambem que a auditoria da O5 cita "v4.3.4" referindo-se a de 08/09, e
que as margens nao mudaram entre as duas - a conferencia segue valida.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012rBhhYMg4csfyvEFcZnaje
</commit_message>
<xml_diff>
--- a/dados/Planilha_Mestra_Winnet_v4_3_4.xlsx
+++ b/dados/Planilha_Mestra_Winnet_v4_3_4.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="16380" windowHeight="8190" tabRatio="500" activeTab="3"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7755" tabRatio="500" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="LEIA-ME" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1837" uniqueCount="558">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1898" uniqueCount="562">
   <si>
     <t>PLANILHA MESTRA WINNET — precificação, margem e frete em um lugar só</t>
   </si>
@@ -1709,6 +1709,18 @@
   </si>
   <si>
     <t>SKUs</t>
+  </si>
+  <si>
+    <t>DEVOLUÇÃO</t>
+  </si>
+  <si>
+    <t>STATUS</t>
+  </si>
+  <si>
+    <t>VÁLIDO</t>
+  </si>
+  <si>
+    <t>702-8393958-4950640 · devolução aprovada 09/09</t>
   </si>
 </sst>
 </file>
@@ -1939,7 +1951,29 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="3">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
@@ -13753,7 +13787,7 @@
         <v>814.08</v>
       </c>
       <c r="I199" s="12">
-        <f t="shared" ref="I199:I262" si="19">IF(OR(G199="",H199=""),"",G199/H199)</f>
+        <f t="shared" ref="I199:I232" si="19">IF(OR(G199="",H199=""),"",G199/H199)</f>
         <v>0.13562549135220126</v>
       </c>
       <c r="J199" s="13">
@@ -13765,19 +13799,19 @@
         <v>233</v>
       </c>
       <c r="L199" s="13">
-        <f t="shared" ref="L199:L262" si="20">IF(OR(J199="",K199=""),"",J199-K199)</f>
+        <f t="shared" ref="L199:L232" si="20">IF(OR(J199="",K199=""),"",J199-K199)</f>
         <v>0</v>
       </c>
       <c r="M199" s="13">
-        <f t="shared" ref="M199:M262" si="21">IF(OR(H199="",F199="",G199=""),"",H199-G199-F199-H199*$B$3+IF(L199="",0,L199))</f>
+        <f t="shared" ref="M199:M232" si="21">IF(OR(H199="",F199="",G199=""),"",H199-G199-F199-H199*$B$3+IF(L199="",0,L199))</f>
         <v>222.09200000000004</v>
       </c>
       <c r="N199" s="12">
-        <f t="shared" ref="N199:N262" si="22">IF(OR(M199="",H199=0,H199=""),"",M199/H199)</f>
+        <f t="shared" ref="N199:N232" si="22">IF(OR(M199="",H199=0,H199=""),"",M199/H199)</f>
         <v>0.27281348270440253</v>
       </c>
       <c r="O199" s="22" t="str">
-        <f t="shared" ref="O199:O262" si="23">IF(N199="","",IF(N199&lt;0,"PREJUÍZO",IF(N199&lt;0.1,"CRÍTICO (&lt;10%)",IF(N199&lt;0.15,"ABAIXO DA META (10-15%)",IF(N199&lt;=0.2,"DENTRO DA META (15-20%)","ACIMA DA META (&gt;20%)")))))</f>
+        <f t="shared" ref="O199:O232" si="23">IF(N199="","",IF(N199&lt;0,"PREJUÍZO",IF(N199&lt;0.1,"CRÍTICO (&lt;10%)",IF(N199&lt;0.15,"ABAIXO DA META (10-15%)",IF(N199&lt;=0.2,"DENTRO DA META (15-20%)","ACIMA DA META (&gt;20%)")))))</f>
         <v>ACIMA DA META (&gt;20%)</v>
       </c>
       <c r="P199" s="23"/>
@@ -15681,7 +15715,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:R117"/>
+  <dimension ref="A1:S117"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11" style="1" customWidth="1"/>
@@ -15701,19 +15735,20 @@
     <col min="16" max="16" width="24" style="1" customWidth="1"/>
     <col min="17" max="17" width="26" style="1" customWidth="1"/>
     <col min="18" max="18" width="11" style="1" customWidth="1"/>
+    <col min="19" max="19" width="13.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:19" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>188</v>
       </c>
     </row>
-    <row r="2" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
         <v>189</v>
       </c>
     </row>
-    <row r="3" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>190</v>
       </c>
@@ -15727,7 +15762,7 @@
         <v>0.13500000000000001</v>
       </c>
     </row>
-    <row r="5" spans="1:18" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:19" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="18" t="s">
         <v>192</v>
       </c>
@@ -15782,8 +15817,11 @@
       <c r="R5" s="18" t="s">
         <v>205</v>
       </c>
-    </row>
-    <row r="6" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="S5" s="18" t="s">
+        <v>559</v>
+      </c>
+    </row>
+    <row r="6" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="32">
         <v>46228</v>
       </c>
@@ -15843,8 +15881,11 @@
       <c r="R6" s="19" t="s">
         <v>207</v>
       </c>
-    </row>
-    <row r="7" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="S6" t="s">
+        <v>560</v>
+      </c>
+    </row>
+    <row r="7" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="32">
         <v>46236</v>
       </c>
@@ -15907,8 +15948,11 @@
       <c r="R7" s="19" t="s">
         <v>210</v>
       </c>
-    </row>
-    <row r="8" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="S7" t="s">
+        <v>560</v>
+      </c>
+    </row>
+    <row r="8" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="32">
         <v>46234</v>
       </c>
@@ -15971,8 +16015,11 @@
       <c r="R8" s="19" t="s">
         <v>210</v>
       </c>
-    </row>
-    <row r="9" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="S8" t="s">
+        <v>560</v>
+      </c>
+    </row>
+    <row r="9" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="32">
         <v>46233</v>
       </c>
@@ -16033,8 +16080,11 @@
       <c r="R9" s="19" t="s">
         <v>207</v>
       </c>
-    </row>
-    <row r="10" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="S9" t="s">
+        <v>560</v>
+      </c>
+    </row>
+    <row r="10" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="32">
         <v>46186</v>
       </c>
@@ -16094,8 +16144,11 @@
       <c r="R10" s="19" t="s">
         <v>207</v>
       </c>
-    </row>
-    <row r="11" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="S10" t="s">
+        <v>560</v>
+      </c>
+    </row>
+    <row r="11" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="32">
         <v>46192</v>
       </c>
@@ -16157,8 +16210,11 @@
       <c r="R11" s="19" t="s">
         <v>210</v>
       </c>
-    </row>
-    <row r="12" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="S11" t="s">
+        <v>560</v>
+      </c>
+    </row>
+    <row r="12" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="32">
         <v>46195</v>
       </c>
@@ -16218,8 +16274,11 @@
       <c r="R12" s="19" t="s">
         <v>207</v>
       </c>
-    </row>
-    <row r="13" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="S12" t="s">
+        <v>560</v>
+      </c>
+    </row>
+    <row r="13" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="32">
         <v>46195</v>
       </c>
@@ -16281,8 +16340,11 @@
       <c r="R13" s="19" t="s">
         <v>210</v>
       </c>
-    </row>
-    <row r="14" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="S13" t="s">
+        <v>560</v>
+      </c>
+    </row>
+    <row r="14" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="32">
         <v>46197</v>
       </c>
@@ -16343,8 +16405,11 @@
       <c r="R14" s="19" t="s">
         <v>210</v>
       </c>
-    </row>
-    <row r="15" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="S14" t="s">
+        <v>560</v>
+      </c>
+    </row>
+    <row r="15" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="32">
         <v>46198</v>
       </c>
@@ -16406,8 +16471,11 @@
       <c r="R15" s="19" t="s">
         <v>210</v>
       </c>
-    </row>
-    <row r="16" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="S15" t="s">
+        <v>560</v>
+      </c>
+    </row>
+    <row r="16" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="32">
         <v>46199</v>
       </c>
@@ -16470,8 +16538,11 @@
       <c r="R16" s="19" t="s">
         <v>207</v>
       </c>
-    </row>
-    <row r="17" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="S16" t="s">
+        <v>560</v>
+      </c>
+    </row>
+    <row r="17" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="32">
         <v>46202</v>
       </c>
@@ -16533,8 +16604,11 @@
       <c r="R17" s="19" t="s">
         <v>210</v>
       </c>
-    </row>
-    <row r="18" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="S17" t="s">
+        <v>560</v>
+      </c>
+    </row>
+    <row r="18" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="32">
         <v>46202</v>
       </c>
@@ -16599,8 +16673,11 @@
       <c r="R18" s="19" t="s">
         <v>210</v>
       </c>
-    </row>
-    <row r="19" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="S18" t="s">
+        <v>560</v>
+      </c>
+    </row>
+    <row r="19" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="32">
         <v>46205</v>
       </c>
@@ -16663,8 +16740,11 @@
       <c r="R19" s="19" t="s">
         <v>207</v>
       </c>
-    </row>
-    <row r="20" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="S19" t="s">
+        <v>560</v>
+      </c>
+    </row>
+    <row r="20" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="32">
         <v>46205</v>
       </c>
@@ -16725,8 +16805,11 @@
       <c r="R20" s="19" t="s">
         <v>210</v>
       </c>
-    </row>
-    <row r="21" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="S20" t="s">
+        <v>560</v>
+      </c>
+    </row>
+    <row r="21" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="32">
         <v>46205</v>
       </c>
@@ -16787,8 +16870,11 @@
       <c r="R21" s="19" t="s">
         <v>210</v>
       </c>
-    </row>
-    <row r="22" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="S21" t="s">
+        <v>560</v>
+      </c>
+    </row>
+    <row r="22" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="32">
         <v>46206</v>
       </c>
@@ -16850,8 +16936,11 @@
       <c r="R22" s="19" t="s">
         <v>207</v>
       </c>
-    </row>
-    <row r="23" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="S22" t="s">
+        <v>560</v>
+      </c>
+    </row>
+    <row r="23" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="32">
         <v>46207</v>
       </c>
@@ -16914,8 +17003,11 @@
       <c r="R23" s="19" t="s">
         <v>207</v>
       </c>
-    </row>
-    <row r="24" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="S23" t="s">
+        <v>560</v>
+      </c>
+    </row>
+    <row r="24" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="32">
         <v>46211</v>
       </c>
@@ -16977,8 +17069,11 @@
       <c r="R24" s="19" t="s">
         <v>210</v>
       </c>
-    </row>
-    <row r="25" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="S24" t="s">
+        <v>560</v>
+      </c>
+    </row>
+    <row r="25" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="32">
         <v>46212</v>
       </c>
@@ -17041,8 +17136,11 @@
       <c r="R25" s="19" t="s">
         <v>210</v>
       </c>
-    </row>
-    <row r="26" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="S25" t="s">
+        <v>560</v>
+      </c>
+    </row>
+    <row r="26" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="32">
         <v>46212</v>
       </c>
@@ -17105,8 +17203,11 @@
       <c r="R26" s="19" t="s">
         <v>210</v>
       </c>
-    </row>
-    <row r="27" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="S26" t="s">
+        <v>560</v>
+      </c>
+    </row>
+    <row r="27" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="32">
         <v>46223</v>
       </c>
@@ -17170,8 +17271,11 @@
       <c r="R27" s="19" t="s">
         <v>210</v>
       </c>
-    </row>
-    <row r="28" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="S27" t="s">
+        <v>560</v>
+      </c>
+    </row>
+    <row r="28" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="32">
         <v>46224</v>
       </c>
@@ -17236,8 +17340,11 @@
       <c r="R28" s="19" t="s">
         <v>210</v>
       </c>
-    </row>
-    <row r="29" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="S28" t="s">
+        <v>560</v>
+      </c>
+    </row>
+    <row r="29" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="32">
         <v>46225</v>
       </c>
@@ -17301,8 +17408,11 @@
       <c r="R29" s="19" t="s">
         <v>210</v>
       </c>
-    </row>
-    <row r="30" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="S29" t="s">
+        <v>560</v>
+      </c>
+    </row>
+    <row r="30" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="32">
         <v>46225</v>
       </c>
@@ -17365,8 +17475,11 @@
       <c r="R30" s="19" t="s">
         <v>210</v>
       </c>
-    </row>
-    <row r="31" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="S30" t="s">
+        <v>560</v>
+      </c>
+    </row>
+    <row r="31" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="32">
         <v>46225</v>
       </c>
@@ -17429,8 +17542,11 @@
       <c r="R31" s="19" t="s">
         <v>210</v>
       </c>
-    </row>
-    <row r="32" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="S31" t="s">
+        <v>560</v>
+      </c>
+    </row>
+    <row r="32" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="32">
         <v>46238</v>
       </c>
@@ -17495,8 +17611,11 @@
       <c r="R32" s="19" t="s">
         <v>210</v>
       </c>
-    </row>
-    <row r="33" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="S32" t="s">
+        <v>560</v>
+      </c>
+    </row>
+    <row r="33" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="32">
         <v>46239</v>
       </c>
@@ -17559,8 +17678,11 @@
       <c r="R33" s="19" t="s">
         <v>207</v>
       </c>
-    </row>
-    <row r="34" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="S33" t="s">
+        <v>560</v>
+      </c>
+    </row>
+    <row r="34" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="32">
         <v>46240</v>
       </c>
@@ -17623,8 +17745,11 @@
       <c r="R34" s="19" t="s">
         <v>210</v>
       </c>
-    </row>
-    <row r="35" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="S34" t="s">
+        <v>560</v>
+      </c>
+    </row>
+    <row r="35" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="32">
         <v>46240</v>
       </c>
@@ -17687,8 +17812,11 @@
       <c r="R35" s="19" t="s">
         <v>210</v>
       </c>
-    </row>
-    <row r="36" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="S35" t="s">
+        <v>560</v>
+      </c>
+    </row>
+    <row r="36" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="32">
         <v>46241</v>
       </c>
@@ -17749,8 +17877,11 @@
       </c>
       <c r="Q36" s="19"/>
       <c r="R36" s="19"/>
-    </row>
-    <row r="37" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="S36" t="s">
+        <v>560</v>
+      </c>
+    </row>
+    <row r="37" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="32">
         <v>46242</v>
       </c>
@@ -17809,8 +17940,11 @@
       </c>
       <c r="Q37" s="19"/>
       <c r="R37" s="19"/>
-    </row>
-    <row r="38" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="S37" t="s">
+        <v>560</v>
+      </c>
+    </row>
+    <row r="38" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="32">
         <v>46242</v>
       </c>
@@ -17869,8 +18003,11 @@
       </c>
       <c r="Q38" s="19"/>
       <c r="R38" s="19"/>
-    </row>
-    <row r="39" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="S38" t="s">
+        <v>560</v>
+      </c>
+    </row>
+    <row r="39" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="32">
         <v>46245</v>
       </c>
@@ -17931,8 +18068,11 @@
       </c>
       <c r="Q39" s="19"/>
       <c r="R39" s="19"/>
-    </row>
-    <row r="40" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="S39" t="s">
+        <v>560</v>
+      </c>
+    </row>
+    <row r="40" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="32">
         <v>46245</v>
       </c>
@@ -17991,8 +18131,11 @@
       </c>
       <c r="Q40" s="19"/>
       <c r="R40" s="19"/>
-    </row>
-    <row r="41" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="S40" t="s">
+        <v>560</v>
+      </c>
+    </row>
+    <row r="41" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="32">
         <v>46246</v>
       </c>
@@ -18050,8 +18193,11 @@
       </c>
       <c r="Q41" s="19"/>
       <c r="R41" s="19"/>
-    </row>
-    <row r="42" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="S41" t="s">
+        <v>560</v>
+      </c>
+    </row>
+    <row r="42" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="32">
         <v>46246</v>
       </c>
@@ -18110,8 +18256,11 @@
       </c>
       <c r="Q42" s="19"/>
       <c r="R42" s="19"/>
-    </row>
-    <row r="43" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="S42" t="s">
+        <v>560</v>
+      </c>
+    </row>
+    <row r="43" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="32">
         <v>46248</v>
       </c>
@@ -18170,8 +18319,11 @@
       </c>
       <c r="Q43" s="19"/>
       <c r="R43" s="19"/>
-    </row>
-    <row r="44" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="S43" t="s">
+        <v>560</v>
+      </c>
+    </row>
+    <row r="44" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="32">
         <v>46250</v>
       </c>
@@ -18230,8 +18382,11 @@
       </c>
       <c r="Q44" s="19"/>
       <c r="R44" s="19"/>
-    </row>
-    <row r="45" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="S44" t="s">
+        <v>560</v>
+      </c>
+    </row>
+    <row r="45" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="32">
         <v>46253</v>
       </c>
@@ -18290,8 +18445,11 @@
       </c>
       <c r="Q45" s="19"/>
       <c r="R45" s="19"/>
-    </row>
-    <row r="46" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="S45" t="s">
+        <v>560</v>
+      </c>
+    </row>
+    <row r="46" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="32">
         <v>46254</v>
       </c>
@@ -18352,8 +18510,11 @@
       </c>
       <c r="Q46" s="19"/>
       <c r="R46" s="19"/>
-    </row>
-    <row r="47" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="S46" t="s">
+        <v>560</v>
+      </c>
+    </row>
+    <row r="47" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="32">
         <v>46260</v>
       </c>
@@ -18412,8 +18573,11 @@
       </c>
       <c r="Q47" s="19"/>
       <c r="R47" s="19"/>
-    </row>
-    <row r="48" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="S47" t="s">
+        <v>560</v>
+      </c>
+    </row>
+    <row r="48" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="32">
         <v>46263</v>
       </c>
@@ -18472,8 +18636,11 @@
       </c>
       <c r="Q48" s="19"/>
       <c r="R48" s="19"/>
-    </row>
-    <row r="49" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="S48" t="s">
+        <v>560</v>
+      </c>
+    </row>
+    <row r="49" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="32">
         <v>46264</v>
       </c>
@@ -18532,8 +18699,11 @@
       </c>
       <c r="Q49" s="19"/>
       <c r="R49" s="19"/>
-    </row>
-    <row r="50" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="S49" t="s">
+        <v>560</v>
+      </c>
+    </row>
+    <row r="50" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="32">
         <v>46265</v>
       </c>
@@ -18592,8 +18762,11 @@
       </c>
       <c r="Q50" s="19"/>
       <c r="R50" s="19"/>
-    </row>
-    <row r="51" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="S50" t="s">
+        <v>560</v>
+      </c>
+    </row>
+    <row r="51" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" s="32">
         <v>46265</v>
       </c>
@@ -18652,8 +18825,11 @@
       </c>
       <c r="Q51" s="19"/>
       <c r="R51" s="19"/>
-    </row>
-    <row r="52" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="S51" t="s">
+        <v>560</v>
+      </c>
+    </row>
+    <row r="52" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A52" s="32">
         <v>46265</v>
       </c>
@@ -18712,8 +18888,11 @@
       </c>
       <c r="Q52" s="19"/>
       <c r="R52" s="19"/>
-    </row>
-    <row r="53" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="S52" t="s">
+        <v>560</v>
+      </c>
+    </row>
+    <row r="53" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A53" s="32">
         <v>46266</v>
       </c>
@@ -18772,8 +18951,11 @@
       </c>
       <c r="Q53" s="19"/>
       <c r="R53" s="19"/>
-    </row>
-    <row r="54" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="S53" t="s">
+        <v>560</v>
+      </c>
+    </row>
+    <row r="54" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A54" s="32">
         <v>46267</v>
       </c>
@@ -18830,10 +19012,15 @@
         <f t="shared" si="10"/>
         <v>ACIMA DA META (&gt;20%)</v>
       </c>
-      <c r="Q54" s="19"/>
+      <c r="Q54" s="19" t="s">
+        <v>561</v>
+      </c>
       <c r="R54" s="19"/>
-    </row>
-    <row r="55" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="S54" t="s">
+        <v>558</v>
+      </c>
+    </row>
+    <row r="55" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A55" s="32">
         <v>46268</v>
       </c>
@@ -18892,8 +19079,11 @@
       </c>
       <c r="Q55" s="19"/>
       <c r="R55" s="19"/>
-    </row>
-    <row r="56" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="S55" t="s">
+        <v>560</v>
+      </c>
+    </row>
+    <row r="56" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56" s="32">
         <v>46270</v>
       </c>
@@ -18952,8 +19142,11 @@
       </c>
       <c r="Q56" s="19"/>
       <c r="R56" s="19"/>
-    </row>
-    <row r="57" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="S56" t="s">
+        <v>560</v>
+      </c>
+    </row>
+    <row r="57" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A57" s="32">
         <v>46272</v>
       </c>
@@ -18970,10 +19163,12 @@
         <f>IF($B57="","",INDEX(Simulador!$D$7:$D$232,MATCH($B57,Simulador!$A$7:$A$232,0)))</f>
         <v>248.75</v>
       </c>
-      <c r="F57" s="20"/>
+      <c r="F57" s="20">
+        <v>24.87</v>
+      </c>
       <c r="G57" s="13">
         <f t="shared" si="6"/>
-        <v>248.75</v>
+        <v>223.88</v>
       </c>
       <c r="H57" s="8" t="str">
         <f>IF($B57="","",INDEX(Simulador!$B$7:$B$232,MATCH($B57,Simulador!$A$7:$A$232,0)))</f>
@@ -18988,7 +19183,7 @@
       </c>
       <c r="K57" s="20">
         <f t="shared" si="11"/>
-        <v>38.97</v>
+        <v>35.61</v>
       </c>
       <c r="L57" s="13">
         <f>IF(OR($B57="",$C57=""),"",$C57*INDEX(Simulador!$F$7:$F$232,MATCH($B57,Simulador!$A$7:$A$232,0)))</f>
@@ -18996,15 +19191,15 @@
       </c>
       <c r="M57" s="13">
         <f t="shared" si="7"/>
-        <v>24.875</v>
+        <v>22.388000000000002</v>
       </c>
       <c r="N57" s="35">
         <f t="shared" si="8"/>
-        <v>74.045000000000002</v>
+        <v>55.021999999999977</v>
       </c>
       <c r="O57" s="12">
         <f t="shared" si="9"/>
-        <v>0.29766834170854273</v>
+        <v>0.24576558870823645</v>
       </c>
       <c r="P57" s="22" t="str">
         <f t="shared" si="10"/>
@@ -19012,108 +19207,141 @@
       </c>
       <c r="Q57" s="19"/>
       <c r="R57" s="19"/>
-    </row>
-    <row r="58" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A58" s="32"/>
-      <c r="B58" s="19"/>
-      <c r="C58" s="19"/>
-      <c r="D58" s="19"/>
-      <c r="E58" s="20" t="str">
+      <c r="S57" t="s">
+        <v>560</v>
+      </c>
+    </row>
+    <row r="58" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A58" s="32">
+        <v>46273</v>
+      </c>
+      <c r="B58" s="19" t="s">
+        <v>126</v>
+      </c>
+      <c r="C58" s="19">
+        <v>2</v>
+      </c>
+      <c r="D58" s="19" t="s">
+        <v>410</v>
+      </c>
+      <c r="E58" s="20">
         <f>IF($B58="","",INDEX(Simulador!$D$7:$D$232,MATCH($B58,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
-      </c>
-      <c r="F58" s="20"/>
-      <c r="G58" s="13" t="str">
+        <v>167.89</v>
+      </c>
+      <c r="F58" s="20">
+        <v>33.58</v>
+      </c>
+      <c r="G58" s="13">
         <f t="shared" si="6"/>
-        <v/>
+        <v>302.2</v>
       </c>
       <c r="H58" s="8" t="str">
         <f>IF($B58="","",INDEX(Simulador!$B$7:$B$232,MATCH($B58,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
-      </c>
-      <c r="I58" s="13" t="str">
+        <v>Pequenos</v>
+      </c>
+      <c r="I58" s="13">
         <f>IF(OR(H58="",$D58=""),"",INDEX(Ref_Frete!$B$2:$G$54,MATCH($D58,Ref_Frete!$A$2:$A$54,0),IF(H58="Pequenos",2,IF(H58="Medios",4,6))))</f>
-        <v/>
-      </c>
-      <c r="J58" s="20"/>
-      <c r="K58" s="20" t="str">
+        <v>29.9</v>
+      </c>
+      <c r="J58" s="20">
+        <v>23.41</v>
+      </c>
+      <c r="K58" s="20">
         <f t="shared" si="11"/>
-        <v/>
-      </c>
-      <c r="L58" s="13" t="str">
+        <v>44.83</v>
+      </c>
+      <c r="L58" s="13">
         <f>IF(OR($B58="",$C58=""),"",$C58*INDEX(Simulador!$F$7:$F$232,MATCH($B58,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
-      </c>
-      <c r="M58" s="13" t="str">
+        <v>169.58</v>
+      </c>
+      <c r="M58" s="13">
         <f t="shared" si="7"/>
-        <v/>
-      </c>
-      <c r="N58" s="35" t="str">
+        <v>30.22</v>
+      </c>
+      <c r="N58" s="35">
         <f t="shared" si="8"/>
-        <v/>
-      </c>
-      <c r="O58" s="12" t="str">
+        <v>64.059999999999945</v>
+      </c>
+      <c r="O58" s="12">
         <f t="shared" si="9"/>
-        <v/>
+        <v>0.21197882197220366</v>
       </c>
       <c r="P58" s="22" t="str">
         <f t="shared" si="10"/>
-        <v/>
+        <v>ACIMA DA META (&gt;20%)</v>
       </c>
       <c r="Q58" s="19"/>
       <c r="R58" s="19"/>
-    </row>
-    <row r="59" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A59" s="32"/>
-      <c r="B59" s="19"/>
-      <c r="C59" s="19"/>
-      <c r="D59" s="19"/>
-      <c r="E59" s="20" t="str">
+      <c r="S58" t="s">
+        <v>560</v>
+      </c>
+    </row>
+    <row r="59" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A59" s="32">
+        <v>46273</v>
+      </c>
+      <c r="B59" s="19" t="s">
+        <v>126</v>
+      </c>
+      <c r="C59" s="19">
+        <v>1</v>
+      </c>
+      <c r="D59" s="19" t="s">
+        <v>213</v>
+      </c>
+      <c r="E59" s="20">
         <f>IF($B59="","",INDEX(Simulador!$D$7:$D$232,MATCH($B59,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
-      </c>
-      <c r="F59" s="20"/>
-      <c r="G59" s="13" t="str">
+        <v>167.89</v>
+      </c>
+      <c r="F59" s="20">
+        <v>16.79</v>
+      </c>
+      <c r="G59" s="13">
         <f t="shared" si="6"/>
-        <v/>
+        <v>151.1</v>
       </c>
       <c r="H59" s="8" t="str">
         <f>IF($B59="","",INDEX(Simulador!$B$7:$B$232,MATCH($B59,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
-      </c>
-      <c r="I59" s="13" t="str">
+        <v>Pequenos</v>
+      </c>
+      <c r="I59" s="13">
         <f>IF(OR(H59="",$D59=""),"",INDEX(Ref_Frete!$B$2:$G$54,MATCH($D59,Ref_Frete!$A$2:$A$54,0),IF(H59="Pequenos",2,IF(H59="Medios",4,6))))</f>
-        <v/>
-      </c>
-      <c r="J59" s="20"/>
-      <c r="K59" s="20" t="str">
+        <v>24.9</v>
+      </c>
+      <c r="J59" s="20">
+        <v>14.22</v>
+      </c>
+      <c r="K59" s="20">
         <f t="shared" si="11"/>
-        <v/>
-      </c>
-      <c r="L59" s="13" t="str">
+        <v>23.76</v>
+      </c>
+      <c r="L59" s="13">
         <f>IF(OR($B59="",$C59=""),"",$C59*INDEX(Simulador!$F$7:$F$232,MATCH($B59,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
-      </c>
-      <c r="M59" s="13" t="str">
+        <v>84.79</v>
+      </c>
+      <c r="M59" s="13">
         <f t="shared" si="7"/>
-        <v/>
-      </c>
-      <c r="N59" s="35" t="str">
+        <v>15.11</v>
+      </c>
+      <c r="N59" s="35">
         <f t="shared" si="8"/>
-        <v/>
-      </c>
-      <c r="O59" s="12" t="str">
+        <v>38.120000000000005</v>
+      </c>
+      <c r="O59" s="12">
         <f t="shared" si="9"/>
-        <v/>
+        <v>0.25228325612177371</v>
       </c>
       <c r="P59" s="22" t="str">
         <f t="shared" si="10"/>
-        <v/>
+        <v>ACIMA DA META (&gt;20%)</v>
       </c>
       <c r="Q59" s="19"/>
       <c r="R59" s="19"/>
-    </row>
-    <row r="60" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="S59" t="s">
+        <v>560</v>
+      </c>
+    </row>
+    <row r="60" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A60" s="32"/>
       <c r="B60" s="19"/>
       <c r="C60" s="19"/>
@@ -19162,8 +19390,11 @@
       </c>
       <c r="Q60" s="19"/>
       <c r="R60" s="19"/>
-    </row>
-    <row r="61" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="S60" t="s">
+        <v>560</v>
+      </c>
+    </row>
+    <row r="61" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A61" s="32"/>
       <c r="B61" s="19"/>
       <c r="C61" s="19"/>
@@ -19213,7 +19444,7 @@
       <c r="Q61" s="19"/>
       <c r="R61" s="19"/>
     </row>
-    <row r="62" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A62" s="32"/>
       <c r="B62" s="19"/>
       <c r="C62" s="19"/>
@@ -19263,7 +19494,7 @@
       <c r="Q62" s="19"/>
       <c r="R62" s="19"/>
     </row>
-    <row r="63" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A63" s="32"/>
       <c r="B63" s="19"/>
       <c r="C63" s="19"/>
@@ -19313,7 +19544,7 @@
       <c r="Q63" s="19"/>
       <c r="R63" s="19"/>
     </row>
-    <row r="64" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A64" s="32"/>
       <c r="B64" s="19"/>
       <c r="C64" s="19"/>
@@ -21224,7 +21455,7 @@
       </c>
       <c r="F102" s="20"/>
       <c r="G102" s="13" t="str">
-        <f t="shared" ref="G102:G133" si="18">IF(OR($B102="",$C102=""),"",$C102*E102-IF(F102="",0,F102))</f>
+        <f t="shared" ref="G102:G107" si="18">IF(OR($B102="",$C102=""),"",$C102*E102-IF(F102="",0,F102))</f>
         <v/>
       </c>
       <c r="H102" s="8" t="str">
@@ -21249,15 +21480,15 @@
         <v/>
       </c>
       <c r="N102" s="35" t="str">
-        <f t="shared" ref="N102:N133" si="20">IF(OR(G102="",J102=""),"",G102+IF(I102="",0,I102)-J102-K102-L102-M102)</f>
+        <f t="shared" ref="N102:N107" si="20">IF(OR(G102="",J102=""),"",G102+IF(I102="",0,I102)-J102-K102-L102-M102)</f>
         <v/>
       </c>
       <c r="O102" s="12" t="str">
-        <f t="shared" ref="O102:O133" si="21">IF(OR(N102="",G102=0,G102=""),"",N102/G102)</f>
+        <f t="shared" ref="O102:O107" si="21">IF(OR(N102="",G102=0,G102=""),"",N102/G102)</f>
         <v/>
       </c>
       <c r="P102" s="22" t="str">
-        <f t="shared" ref="P102:P133" si="22">IF(O102="","",IF(O102&lt;0,"PREJUÍZO",IF(O102&lt;0.1,"CRÍTICO (&lt;10%)",IF(O102&lt;0.15,"ABAIXO DA META (10-15%)",IF(O102&lt;=0.2,"DENTRO DA META (15-20%)","ACIMA DA META (&gt;20%)")))))</f>
+        <f t="shared" ref="P102:P107" si="22">IF(O102="","",IF(O102&lt;0,"PREJUÍZO",IF(O102&lt;0.1,"CRÍTICO (&lt;10%)",IF(O102&lt;0.15,"ABAIXO DA META (10-15%)",IF(O102&lt;=0.2,"DENTRO DA META (15-20%)","ACIMA DA META (&gt;20%)")))))</f>
         <v/>
       </c>
       <c r="Q102" s="19"/>
@@ -21519,37 +21750,48 @@
       </c>
       <c r="G108" s="39">
         <f>SUM(G6:G107)</f>
-        <v>22896.250000000011</v>
+        <v>23324.680000000011</v>
       </c>
       <c r="K108" s="39">
         <f>SUM(K6:K107)</f>
-        <v>3480.8000000000006</v>
+        <v>3546.0300000000011</v>
       </c>
       <c r="L108" s="39">
         <f>SUM(L6:L107)</f>
-        <v>12002.130000000001</v>
+        <v>12256.500000000002</v>
       </c>
       <c r="M108" s="39">
         <f>SUM(M6:M107)</f>
-        <v>2289.6250000000005</v>
+        <v>2332.4680000000003</v>
       </c>
       <c r="N108" s="39">
         <f>SUM(N6:N107)</f>
-        <v>5816.7350000000015</v>
+        <v>5899.8920000000007</v>
       </c>
       <c r="O108" s="40">
         <f>IF(G108=0,"",N108/G108)</f>
-        <v>0.25404749686083961</v>
+        <v>0.25294632123570387</v>
       </c>
     </row>
     <row r="117" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A117" s="41"/>
     </row>
   </sheetData>
-  <dataValidations count="1">
+  <conditionalFormatting sqref="S6:S60">
+    <cfRule type="cellIs" dxfId="0" priority="2" operator="equal">
+      <formula>"VÁLIDO"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="1" priority="1" operator="equal">
+      <formula>"DEVOLUÇÃO"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="2">
     <dataValidation type="list" allowBlank="1" sqref="R6:R107">
       <formula1>"Ads,Orgânico,Conferir"</formula1>
       <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="S6:S1048576">
+      <formula1>"VÁLIDO,DEVOLUÇÃO"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>